<commit_message>
docs(submit): 테이블 정의서 작성일 2026-06-22로 정정
</commit_message>
<xml_diff>
--- a/산출물/99_제출파일/테이블_정의서.xlsx
+++ b/산출물/99_제출파일/테이블_정의서.xlsx
@@ -576,7 +576,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>하모니 미니앱 DB · SQLite(node:sqlite, 외부 의존 없음) · 작성 김민혁(Backend) · 근거 apps/api/server.mjs · 2026-06-27</t>
+          <t>하모니 미니앱 DB · SQLite(node:sqlite, 외부 의존 없음) · 작성 김민혁(Backend) · 근거 apps/api/server.mjs · 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D7" s="7" t="n"/>
@@ -1262,7 +1262,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>하모니 미니앱 DB · SQLite(node:sqlite, 외부 의존 없음) · 작성 김민혁(Backend) · 근거 apps/api/server.mjs · 2026-06-27</t>
+          <t>하모니 미니앱 DB · SQLite(node:sqlite, 외부 의존 없음) · 작성 김민혁(Backend) · 근거 apps/api/server.mjs · 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D7" s="7" t="n"/>
@@ -2277,7 +2277,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>하모니 미니앱 DB · SQLite(node:sqlite, 외부 의존 없음) · 작성 김민혁(Backend) · 근거 apps/api/server.mjs · 2026-06-27</t>
+          <t>하모니 미니앱 DB · SQLite(node:sqlite, 외부 의존 없음) · 작성 김민혁(Backend) · 근거 apps/api/server.mjs · 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2349,7 @@
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D7" s="7" t="n"/>
@@ -3088,7 +3088,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>하모니 미니앱 DB · SQLite(node:sqlite, 외부 의존 없음) · 작성 김민혁(Backend) · 근거 apps/api/server.mjs · 2026-06-27</t>
+          <t>하모니 미니앱 DB · SQLite(node:sqlite, 외부 의존 없음) · 작성 김민혁(Backend) · 근거 apps/api/server.mjs · 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3160,7 @@
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D7" s="7" t="n"/>
@@ -3899,7 +3899,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>하모니 미니앱 DB · SQLite(node:sqlite, 외부 의존 없음) · 작성 김민혁(Backend) · 근거 apps/api/server.mjs · 2026-06-27</t>
+          <t>하모니 미니앱 DB · SQLite(node:sqlite, 외부 의존 없음) · 작성 김민혁(Backend) · 근거 apps/api/server.mjs · 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D7" s="7" t="n"/>
@@ -4527,7 +4527,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>하모니 미니앱 DB · SQLite(node:sqlite, 외부 의존 없음) · 작성 김민혁(Backend) · 근거 apps/api/server.mjs · 2026-06-27</t>
+          <t>하모니 미니앱 DB · SQLite(node:sqlite, 외부 의존 없음) · 작성 김민혁(Backend) · 근거 apps/api/server.mjs · 2026-06-22</t>
         </is>
       </c>
     </row>
@@ -4599,7 +4599,7 @@
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D7" s="7" t="n"/>

</xml_diff>